<commit_message>
rol lector y plantillas de importacion
</commit_message>
<xml_diff>
--- a/importaciones/Plantilla Importacion Insumos.xlsx
+++ b/importaciones/Plantilla Importacion Insumos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\inverclinikProject\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE127DDC-5A50-4D48-9AAE-F5D15EBBE3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B4B6F8-C49D-44ED-B6BA-621D81707325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="15" windowWidth="14400" windowHeight="7335" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Lista Insumos</t>
   </si>
@@ -40,6 +40,18 @@
   </si>
   <si>
     <t>Proveedor</t>
+  </si>
+  <si>
+    <t>Stock Minimo</t>
+  </si>
+  <si>
+    <t>Stock Maximo</t>
+  </si>
+  <si>
+    <t>Almacen</t>
+  </si>
+  <si>
+    <t>Adicional</t>
   </si>
 </sst>
 </file>
@@ -391,24 +403,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.140625" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -420,11 +440,23 @@
       </c>
       <c r="D2" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>